<commit_message>
Added RGB-led feature for controller state, added documentation for S200 wind sensor
</commit_message>
<xml_diff>
--- a/finance/20260329_Begroting.xlsx
+++ b/finance/20260329_Begroting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\drasv\github\greenhouse-Controller\finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99F87B4-224A-4490-A910-AD0CD1C4E226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8749C689-FA72-4999-B79E-D0729755804F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1110" windowWidth="25440" windowHeight="15270" xr2:uid="{69D97536-DC5A-4EC7-9137-936378E5A619}"/>
   </bookViews>
@@ -200,9 +200,6 @@
     <t xml:space="preserve"> DS1307 — Real Time Clock IC, I2C / Serial, 4.5–5.5 V, DIP-8 </t>
   </si>
   <si>
-    <t xml:space="preserve"> [Farnell](https://nl.farnell.com/analog-devices/ds1307/real-time-clock/dp/2515369) </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Raltron R38-32.768-12.5 — 32.768 kHz, 20 ppm, 12.5 pF *(min. order 5)* </t>
   </si>
   <si>
@@ -336,6 +333,9 @@
   </si>
   <si>
     <t>Verzendkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> [Farnell](https://nl.farnell.com/analog-devices/ds1307z-t-r/rtc-i2c-serial-5-5v-soic-8/dp/2798723) </t>
   </si>
 </sst>
 </file>
@@ -361,12 +361,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -391,11 +397,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -739,7 +746,7 @@
     <col min="3" max="3" width="33.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="74.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6640625" customWidth="1"/>
+    <col min="6" max="6" width="59.44140625" customWidth="1"/>
     <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="2" bestFit="1" customWidth="1"/>
   </cols>
@@ -749,7 +756,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -772,10 +779,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2">
         <v>6</v>
@@ -795,10 +802,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D3">
         <v>6</v>
@@ -818,10 +825,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D4">
         <v>6</v>
@@ -841,10 +848,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D5">
         <v>8</v>
@@ -864,10 +871,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -887,10 +894,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -910,10 +917,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -933,10 +940,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -956,10 +963,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -979,10 +986,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -1002,10 +1009,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1025,10 +1032,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1048,10 +1055,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1071,10 +1078,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D15">
         <v>3</v>
@@ -1094,10 +1101,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D16">
         <v>2</v>
@@ -1117,10 +1124,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D17">
         <v>10</v>
@@ -1140,10 +1147,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D18">
         <v>10</v>
@@ -1163,10 +1170,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D19">
         <v>10</v>
@@ -1186,10 +1193,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1209,10 +1216,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1232,10 +1239,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -1243,7 +1250,7 @@
       <c r="E22" t="s">
         <v>44</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="4" t="s">
         <v>45</v>
       </c>
       <c r="G22" s="1">
@@ -1255,10 +1262,10 @@
         <v>23</v>
       </c>
       <c r="B23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1278,10 +1285,10 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1301,10 +1308,10 @@
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -1312,8 +1319,8 @@
       <c r="E25" t="s">
         <v>53</v>
       </c>
-      <c r="F25" t="s">
-        <v>54</v>
+      <c r="F25" s="4" t="s">
+        <v>99</v>
       </c>
       <c r="G25" s="1">
         <v>9.14</v>
@@ -1324,19 +1331,19 @@
         <v>26</v>
       </c>
       <c r="B26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D26">
         <v>1</v>
       </c>
       <c r="E26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="F26" t="s">
-        <v>56</v>
       </c>
       <c r="G26" s="1">
         <v>0.68</v>
@@ -1347,19 +1354,19 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D27">
         <v>1</v>
       </c>
       <c r="E27" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" t="s">
         <v>57</v>
-      </c>
-      <c r="F27" t="s">
-        <v>58</v>
       </c>
       <c r="G27" s="1">
         <v>0.5</v>
@@ -1370,22 +1377,22 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C28" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D28">
         <v>4</v>
       </c>
       <c r="E28" t="s">
+        <v>58</v>
+      </c>
+      <c r="F28" t="s">
         <v>59</v>
       </c>
-      <c r="F28" t="s">
-        <v>60</v>
-      </c>
       <c r="G28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1393,19 +1400,19 @@
         <v>29</v>
       </c>
       <c r="B29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D29">
         <v>4</v>
       </c>
       <c r="E29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G29" s="1">
         <v>6</v>
@@ -1416,19 +1423,19 @@
         <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D30">
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F30" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G30" s="1">
         <v>60</v>
@@ -1439,16 +1446,16 @@
         <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C31" t="s">
+        <v>95</v>
+      </c>
+      <c r="E31" t="s">
         <v>96</v>
       </c>
-      <c r="E31" t="s">
-        <v>97</v>
-      </c>
       <c r="F31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G31" s="2">
         <f>0.2*SUM(G2:G30)</f>
@@ -1460,13 +1467,13 @@
         <v>32</v>
       </c>
       <c r="C32" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G32" s="2">
         <v>40</v>
@@ -1476,12 +1483,12 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="E34" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G34" s="2">
         <f>SUM(G2:G33)</f>
@@ -1493,7 +1500,7 @@
         <v>22</v>
       </c>
       <c r="B37" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C37" t="s">
         <v>46</v>

</xml_diff>